<commit_message>
SYCHECF winter peak updates
</commit_message>
<xml_diff>
--- a/InputData/web-app/OCCF/Output Currency Conversion Factors.xlsx
+++ b/InputData/web-app/OCCF/Output Currency Conversion Factors.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28715"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MeganMahajan\Documents\eps-us\InputData\web-app\OCCF\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Rachel Goldstein\Desktop\EPS Models\Mexico EPS\InputData\web-app\OCCF\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="20" documentId="13_ncr:1_{6B6FEF58-08A4-48D5-A6A7-14155C535D30}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CEC4F9A2-C634-4475-8D19-9008F6E7DE94}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CCA2F14E-082D-4A6C-8CE3-BEBFA3E084DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="48015" yWindow="2685" windowWidth="18480" windowHeight="12900" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -83,21 +83,12 @@
     <t>Large Output Currency Unit</t>
   </si>
   <si>
-    <t>billion 2023 Mexican Pesos (MXN)</t>
-  </si>
-  <si>
     <t>Medium Output Currency Unit</t>
   </si>
   <si>
-    <t>million 2023 Mexican Pesos (MXN)</t>
-  </si>
-  <si>
     <t>Small Output Currency Unit</t>
   </si>
   <si>
-    <t>2023 Mexican Pesos (MXN)</t>
-  </si>
-  <si>
     <t>2023 MXN per 2012 USD</t>
   </si>
   <si>
@@ -132,13 +123,22 @@
   </si>
   <si>
     <t>One Small Output Currency Unit</t>
+  </si>
+  <si>
+    <t>2023 Mexican Pesos (MXN$)</t>
+  </si>
+  <si>
+    <t>million 2023 Mexican Pesos (MXN$)</t>
+  </si>
+  <si>
+    <t>billion 2023 Mexican Pesos (MXN$)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -496,27 +496,27 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B36"/>
-  <sheetFormatPr defaultRowHeight="14.45"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="26.28515625" customWidth="1"/>
+    <col min="2" max="2" width="26.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:2">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="1:2">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
         <v>3</v>
       </c>
@@ -524,132 +524,132 @@
         <v>4</v>
       </c>
     </row>
-    <row r="7" spans="1:2">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:2">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="9" spans="1:2">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="10" spans="1:2">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="11" spans="1:2">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="12" spans="1:2">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="13" spans="1:2">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="15" spans="1:2">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="17" spans="1:2">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A17" s="4" t="s">
         <v>13</v>
       </c>
       <c r="B17" s="5"/>
     </row>
-    <row r="18" spans="1:2">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A20" s="4" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="20" spans="1:2">
-      <c r="A20" s="4" t="s">
+      <c r="B20" s="5"/>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A23" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="B20" s="5"/>
-    </row>
-    <row r="21" spans="1:2">
-      <c r="A21" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2">
-      <c r="A23" s="4" t="s">
-        <v>17</v>
-      </c>
       <c r="B23" s="5"/>
     </row>
-    <row r="24" spans="1:2">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="26" spans="1:2">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A26">
         <f>1/(1/A29/A28)</f>
         <v>4.2542803263516484E-2</v>
       </c>
       <c r="B26" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="28" spans="1:2" ht="15">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A28">
         <v>5.6460000000000003E-2</v>
       </c>
       <c r="B28" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="29" spans="1:2">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A29">
         <v>0.75350342301658668</v>
       </c>
       <c r="B29" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B31" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B32" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="33" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B33" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="31" spans="1:2">
-      <c r="B31" t="s">
+    <row r="34" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B34" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="32" spans="1:2">
-      <c r="B32" t="s">
+    <row r="35" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B35" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="33" spans="2:2">
-      <c r="B33" t="s">
+    <row r="36" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B36" t="s">
         <v>24</v>
-      </c>
-    </row>
-    <row r="34" spans="2:2">
-      <c r="B34" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="35" spans="2:2">
-      <c r="B35" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="36" spans="2:2">
-      <c r="B36" t="s">
-        <v>27</v>
       </c>
     </row>
   </sheetData>
@@ -664,19 +664,19 @@
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="14.45"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="31.28515625" customWidth="1"/>
+    <col min="2" max="2" width="31.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="B1" s="3" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="B2" s="2">
         <f>10^9*About!$A$29</f>
@@ -694,19 +694,19 @@
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="14.45"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="31.28515625" customWidth="1"/>
+    <col min="2" max="2" width="31.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="B1" s="3" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="B2" s="6">
         <f>10^6*About!$A$29</f>
@@ -724,19 +724,19 @@
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="14.45"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="31.28515625" customWidth="1"/>
+    <col min="2" max="2" width="31.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="B1" s="3" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="B2">
         <f>1*About!A29</f>
@@ -749,21 +749,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101009A9DAB439B36DB4795F39C4E722C7BC4" ma:contentTypeVersion="4" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="44674c89fa9bc5e97a878a6680c46188">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="79748b23-d81a-423e-9112-21109dc864e6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="447839a363ea5a12024b5bf1ab53ed90" ns2:_="">
     <xsd:import namespace="79748b23-d81a-423e-9112-21109dc864e6"/>
@@ -907,14 +892,52 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{344CD8FC-E2A0-4EE7-AFF9-D02002E55732}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{17CFF595-95A3-4F62-9F72-80600493741F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="79748b23-d81a-423e-9112-21109dc864e6"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FA9BC424-9974-4873-AEBE-9FBC926B8FEA}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FA9BC424-9974-4873-AEBE-9FBC926B8FEA}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{17CFF595-95A3-4F62-9F72-80600493741F}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{344CD8FC-E2A0-4EE7-AFF9-D02002E55732}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>